<commit_message>
data: 更新 2026-05 (TT=195.694 Kwai=61.504)
</commit_message>
<xml_diff>
--- a/docs/data/巴西数据底稿_2026-05.xlsx
+++ b/docs/data/巴西数据底稿_2026-05.xlsx
@@ -516,46 +516,46 @@
     </row>
     <row r="2">
       <c r="B2" t="n">
-        <v>348.84</v>
+        <v>404.78</v>
       </c>
       <c r="C2" t="n">
-        <v>321.59</v>
+        <v>392.53</v>
       </c>
       <c r="D2" t="n">
-        <v>1.15</v>
+        <v>1.22</v>
       </c>
       <c r="E2" t="n">
-        <v>257.48</v>
+        <v>271.03</v>
       </c>
       <c r="F2" t="n">
-        <v>8</v>
+        <v>9.35</v>
       </c>
       <c r="G2" t="n">
-        <v>87.76000000000001</v>
+        <v>110.45</v>
       </c>
       <c r="H2" t="n">
-        <v>0.43</v>
+        <v>0.6</v>
       </c>
       <c r="I2" t="n">
-        <v>6</v>
+        <v>7.34</v>
       </c>
       <c r="J2" t="n">
-        <v>96.95999999999999</v>
+        <v>99.91</v>
       </c>
       <c r="K2" t="n">
-        <v>15.8</v>
+        <v>20.69</v>
       </c>
       <c r="L2" t="n">
-        <v>107.72</v>
+        <v>105.82</v>
       </c>
       <c r="M2" t="n">
-        <v>25.02</v>
+        <v>33.15</v>
       </c>
       <c r="N2" t="n">
-        <v>33.59</v>
+        <v>45.84</v>
       </c>
       <c r="O2" t="n">
-        <v>41.61</v>
+        <v>42.51</v>
       </c>
     </row>
     <row r="3">
@@ -565,7 +565,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>218.098</v>
+        <v>261.451</v>
       </c>
     </row>
     <row r="4">
@@ -575,7 +575,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>115.283</v>
+        <v>125.571</v>
       </c>
     </row>
     <row r="5">
@@ -585,7 +585,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.897</v>
+        <v>4.673</v>
       </c>
     </row>
     <row r="6">
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2.087</v>
+        <v>2.609</v>
       </c>
     </row>
     <row r="7">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.8129999999999999</v>
+        <v>1.823</v>
       </c>
     </row>
     <row r="9">
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>62.076</v>
+        <v>132.957</v>
       </c>
     </row>
     <row r="11">
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2.319</v>
+        <v>2.374</v>
       </c>
     </row>
     <row r="13">
@@ -665,7 +665,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.503</v>
+        <v>0.533</v>
       </c>
     </row>
     <row r="16">
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.282</v>
+        <v>0.295</v>
       </c>
     </row>
     <row r="17">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.263</v>
+        <v>0.279</v>
       </c>
     </row>
     <row r="18">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.104</v>
+        <v>0.109</v>
       </c>
     </row>
     <row r="20">
@@ -705,7 +705,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>226.164</v>
+        <v>236.016</v>
       </c>
     </row>
     <row r="21">
@@ -715,7 +715,7 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>11.696</v>
+        <v>14.243</v>
       </c>
     </row>
     <row r="22">
@@ -725,27 +725,27 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>3.831</v>
+        <v>3.59</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>YouTube Kids</t>
+          <t>Amazon Prime Video</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>2.729</v>
+        <v>2.883</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Amazon Prime Video</t>
+          <t>YouTube Kids</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>2.445</v>
+        <v>2.742</v>
       </c>
     </row>
     <row r="26">
@@ -755,7 +755,7 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.401</v>
+        <v>4.198</v>
       </c>
     </row>
     <row r="27">
@@ -765,7 +765,7 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.04</v>
+        <v>2.368</v>
       </c>
     </row>
     <row r="28">
@@ -775,7 +775,7 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>0.835</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="29">
@@ -785,7 +785,7 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>0.784</v>
+        <v>0.762</v>
       </c>
     </row>
     <row r="30">
@@ -795,7 +795,7 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>0.398</v>
+        <v>0.499</v>
       </c>
     </row>
     <row r="32">
@@ -805,7 +805,7 @@
         </is>
       </c>
       <c r="G32" t="n">
-        <v>63.053</v>
+        <v>83.248</v>
       </c>
     </row>
     <row r="33">
@@ -815,7 +815,7 @@
         </is>
       </c>
       <c r="G33" t="n">
-        <v>9.67</v>
+        <v>11.593</v>
       </c>
     </row>
     <row r="34">
@@ -825,7 +825,7 @@
         </is>
       </c>
       <c r="G34" t="n">
-        <v>5.933</v>
+        <v>6.049</v>
       </c>
     </row>
     <row r="35">
@@ -835,7 +835,7 @@
         </is>
       </c>
       <c r="G35" t="n">
-        <v>5.826</v>
+        <v>5.878</v>
       </c>
     </row>
     <row r="36">
@@ -845,37 +845,37 @@
         </is>
       </c>
       <c r="G36" t="n">
-        <v>1.711</v>
+        <v>1.952</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Google News</t>
+          <t>G1</t>
         </is>
       </c>
       <c r="H38" t="n">
-        <v>0.082</v>
+        <v>0.123</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Panflix</t>
+          <t>Google News</t>
         </is>
       </c>
       <c r="H39" t="n">
-        <v>0.068</v>
+        <v>0.093</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>G1</t>
+          <t>Panflix</t>
         </is>
       </c>
       <c r="H40" t="n">
-        <v>0.065</v>
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="41">
@@ -885,17 +885,17 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>0.028</v>
+        <v>0.06900000000000001</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Estadao</t>
+          <t>Folha de S.Paulo</t>
         </is>
       </c>
       <c r="H42" t="n">
-        <v>0.028</v>
+        <v>0.019</v>
       </c>
     </row>
     <row r="44">
@@ -905,47 +905,47 @@
         </is>
       </c>
       <c r="I44" t="n">
-        <v>1.436</v>
+        <v>1.748</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>JW Library</t>
+          <t>Kindle</t>
         </is>
       </c>
       <c r="I45" t="n">
-        <v>0.792</v>
+        <v>0.826</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Kindle</t>
+          <t>JW Library</t>
         </is>
       </c>
       <c r="I46" t="n">
-        <v>0.442</v>
+        <v>0.8070000000000001</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>ReadEra by READERA LLC</t>
+          <t>GALATEA</t>
         </is>
       </c>
       <c r="I47" t="n">
-        <v>0.39</v>
+        <v>0.5580000000000001</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Bible</t>
+          <t>ReadEra by READERA LLC</t>
         </is>
       </c>
       <c r="I48" t="n">
-        <v>0.272</v>
+        <v>0.375</v>
       </c>
     </row>
     <row r="50">
@@ -955,7 +955,7 @@
         </is>
       </c>
       <c r="J50" t="n">
-        <v>59.772</v>
+        <v>59.544</v>
       </c>
     </row>
     <row r="51">
@@ -965,7 +965,7 @@
         </is>
       </c>
       <c r="J51" t="n">
-        <v>23.317</v>
+        <v>26.815</v>
       </c>
     </row>
     <row r="52">
@@ -975,7 +975,7 @@
         </is>
       </c>
       <c r="J52" t="n">
-        <v>3.816</v>
+        <v>3.85</v>
       </c>
     </row>
     <row r="53">
@@ -985,7 +985,7 @@
         </is>
       </c>
       <c r="J53" t="n">
-        <v>2.742</v>
+        <v>2.577</v>
       </c>
     </row>
     <row r="54">
@@ -995,7 +995,7 @@
         </is>
       </c>
       <c r="J54" t="n">
-        <v>2.03</v>
+        <v>1.944</v>
       </c>
     </row>
     <row r="56">
@@ -1005,7 +1005,7 @@
         </is>
       </c>
       <c r="K56" t="n">
-        <v>5.783</v>
+        <v>9.939</v>
       </c>
     </row>
     <row r="57">
@@ -1015,7 +1015,7 @@
         </is>
       </c>
       <c r="K57" t="n">
-        <v>4.688</v>
+        <v>4.949</v>
       </c>
     </row>
     <row r="58">
@@ -1025,7 +1025,7 @@
         </is>
       </c>
       <c r="K58" t="n">
-        <v>1.006</v>
+        <v>0.997</v>
       </c>
     </row>
     <row r="59">
@@ -1035,17 +1035,17 @@
         </is>
       </c>
       <c r="K59" t="n">
-        <v>0.633</v>
+        <v>0.616</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Music Player - MP3 Player, Audio Player</t>
+          <t>Deezer</t>
         </is>
       </c>
       <c r="K60" t="n">
-        <v>0.223</v>
+        <v>0.24</v>
       </c>
     </row>
     <row r="62">
@@ -1055,7 +1055,7 @@
         </is>
       </c>
       <c r="L62" t="n">
-        <v>34.819</v>
+        <v>30.737</v>
       </c>
     </row>
     <row r="63">
@@ -1065,7 +1065,7 @@
         </is>
       </c>
       <c r="L63" t="n">
-        <v>6.322</v>
+        <v>6.081</v>
       </c>
     </row>
     <row r="64">
@@ -1075,7 +1075,7 @@
         </is>
       </c>
       <c r="L64" t="n">
-        <v>4.372</v>
+        <v>4.623</v>
       </c>
     </row>
     <row r="65">
@@ -1085,7 +1085,7 @@
         </is>
       </c>
       <c r="L65" t="n">
-        <v>3.67</v>
+        <v>3.285</v>
       </c>
     </row>
     <row r="66">
@@ -1095,7 +1095,7 @@
         </is>
       </c>
       <c r="L66" t="n">
-        <v>1.922</v>
+        <v>2.163</v>
       </c>
     </row>
     <row r="68">
@@ -1105,7 +1105,7 @@
         </is>
       </c>
       <c r="M68" t="n">
-        <v>11.122</v>
+        <v>15.561</v>
       </c>
     </row>
     <row r="69">
@@ -1115,7 +1115,7 @@
         </is>
       </c>
       <c r="M69" t="n">
-        <v>5.73</v>
+        <v>7.125</v>
       </c>
     </row>
     <row r="70">
@@ -1125,7 +1125,7 @@
         </is>
       </c>
       <c r="M70" t="n">
-        <v>2.625</v>
+        <v>3.644</v>
       </c>
     </row>
     <row r="71">
@@ -1135,7 +1135,7 @@
         </is>
       </c>
       <c r="M71" t="n">
-        <v>1.156</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="72">
@@ -1145,7 +1145,7 @@
         </is>
       </c>
       <c r="M72" t="n">
-        <v>0.98</v>
+        <v>1.072</v>
       </c>
     </row>
     <row r="74">
@@ -1155,7 +1155,7 @@
         </is>
       </c>
       <c r="N74" t="n">
-        <v>4.87</v>
+        <v>9.698</v>
       </c>
     </row>
     <row r="75">
@@ -1165,37 +1165,37 @@
         </is>
       </c>
       <c r="N75" t="n">
-        <v>4.181</v>
+        <v>4.952</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Uber Driver</t>
+          <t>99 POP</t>
         </is>
       </c>
       <c r="N76" t="n">
-        <v>2.76</v>
+        <v>3.48</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>99 POP</t>
+          <t>Nubank</t>
         </is>
       </c>
       <c r="N77" t="n">
-        <v>2.675</v>
+        <v>3.053</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Nubank</t>
+          <t>Uber Driver</t>
         </is>
       </c>
       <c r="N78" t="n">
-        <v>2.451</v>
+        <v>2.851</v>
       </c>
     </row>
     <row r="80">
@@ -1205,7 +1205,7 @@
         </is>
       </c>
       <c r="O80" t="n">
-        <v>13.64</v>
+        <v>14.344</v>
       </c>
     </row>
     <row r="81">
@@ -1215,7 +1215,7 @@
         </is>
       </c>
       <c r="O81" t="n">
-        <v>9.956</v>
+        <v>10.377</v>
       </c>
     </row>
     <row r="82">
@@ -1225,7 +1225,7 @@
         </is>
       </c>
       <c r="O82" t="n">
-        <v>5.727</v>
+        <v>5.595</v>
       </c>
     </row>
     <row r="83">
@@ -1235,7 +1235,7 @@
         </is>
       </c>
       <c r="O83" t="n">
-        <v>2.458</v>
+        <v>2.338</v>
       </c>
     </row>
     <row r="84">
@@ -1245,7 +1245,7 @@
         </is>
       </c>
       <c r="O84" t="n">
-        <v>1.89</v>
+        <v>1.761</v>
       </c>
     </row>
     <row r="86">
@@ -1255,40 +1255,40 @@
         </is>
       </c>
       <c r="B86" t="n">
-        <v>7.665</v>
+        <v>8.65</v>
       </c>
       <c r="E86" t="n">
-        <v>10.617</v>
+        <v>11.557</v>
       </c>
       <c r="F86" t="n">
-        <v>0.541</v>
+        <v>0.694</v>
       </c>
       <c r="G86" t="n">
-        <v>1.564</v>
+        <v>1.733</v>
       </c>
       <c r="H86" t="n">
-        <v>0.16</v>
+        <v>0.222</v>
       </c>
       <c r="I86" t="n">
-        <v>2.668</v>
+        <v>3.023</v>
       </c>
       <c r="J86" t="n">
-        <v>5.28</v>
+        <v>5.18</v>
       </c>
       <c r="K86" t="n">
-        <v>3.466</v>
+        <v>3.953</v>
       </c>
       <c r="L86" t="n">
-        <v>56.613</v>
+        <v>58.931</v>
       </c>
       <c r="M86" t="n">
-        <v>3.411</v>
+        <v>4.249</v>
       </c>
       <c r="N86" t="n">
-        <v>16.653</v>
+        <v>21.807</v>
       </c>
       <c r="O86" t="n">
-        <v>7.943</v>
+        <v>8.090999999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Restore confirmed May output and lock historical snapshot
</commit_message>
<xml_diff>
--- a/docs/data/巴西数据底稿_2026-05.xlsx
+++ b/docs/data/巴西数据底稿_2026-05.xlsx
@@ -1,13 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="2026_05" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026_05" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="未分类App" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -516,46 +517,46 @@
     </row>
     <row r="2">
       <c r="B2" t="n">
-        <v>404.78</v>
+        <v>397.08</v>
       </c>
       <c r="C2" t="n">
-        <v>392.53</v>
+        <v>394.85</v>
       </c>
       <c r="D2" t="n">
         <v>1.22</v>
       </c>
       <c r="E2" t="n">
-        <v>271.03</v>
+        <v>273.27</v>
       </c>
       <c r="F2" t="n">
-        <v>9.35</v>
+        <v>9.23</v>
       </c>
       <c r="G2" t="n">
-        <v>110.45</v>
+        <v>113.55</v>
       </c>
       <c r="H2" t="n">
-        <v>0.6</v>
+        <v>0.63</v>
       </c>
       <c r="I2" t="n">
-        <v>7.34</v>
+        <v>7.18</v>
       </c>
       <c r="J2" t="n">
-        <v>99.91</v>
+        <v>97.03</v>
       </c>
       <c r="K2" t="n">
-        <v>20.69</v>
+        <v>21.04</v>
       </c>
       <c r="L2" t="n">
-        <v>105.82</v>
+        <v>127.37</v>
       </c>
       <c r="M2" t="n">
-        <v>33.15</v>
+        <v>31.49</v>
       </c>
       <c r="N2" t="n">
-        <v>45.84</v>
+        <v>48.63</v>
       </c>
       <c r="O2" t="n">
-        <v>42.51</v>
+        <v>43.51</v>
       </c>
     </row>
     <row r="3">
@@ -565,7 +566,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>261.451</v>
+        <v>251.025</v>
       </c>
     </row>
     <row r="4">
@@ -575,7 +576,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>125.571</v>
+        <v>127.6</v>
       </c>
     </row>
     <row r="5">
@@ -585,7 +586,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.673</v>
+        <v>4.809</v>
       </c>
     </row>
     <row r="6">
@@ -595,7 +596,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2.609</v>
+        <v>2.532</v>
       </c>
     </row>
     <row r="7">
@@ -605,7 +606,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1.823</v>
+        <v>1.842</v>
       </c>
     </row>
     <row r="9">
@@ -625,7 +626,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>132.957</v>
+        <v>135.106</v>
       </c>
     </row>
     <row r="11">
@@ -645,7 +646,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2.374</v>
+        <v>2.543</v>
       </c>
     </row>
     <row r="13">
@@ -665,13 +666,13 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.533</v>
+        <v>0.5669999999999999</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Pluto.tv</t>
+          <t>BIGO LIVE</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -681,11 +682,11 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>BIGO LIVE</t>
+          <t>Pluto.tv</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.279</v>
+        <v>0.276</v>
       </c>
     </row>
     <row r="18">
@@ -695,7 +696,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.109</v>
+        <v>0.08599999999999999</v>
       </c>
     </row>
     <row r="20">
@@ -705,7 +706,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>236.016</v>
+        <v>239.136</v>
       </c>
     </row>
     <row r="21">
@@ -715,7 +716,7 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>14.243</v>
+        <v>13.151</v>
       </c>
     </row>
     <row r="22">
@@ -725,7 +726,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>3.59</v>
+        <v>3.718</v>
       </c>
     </row>
     <row r="23">
@@ -735,17 +736,17 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>2.883</v>
+        <v>2.821</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>YouTube Kids</t>
+          <t>Globo Play</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>2.742</v>
+        <v>2.801</v>
       </c>
     </row>
     <row r="26">
@@ -755,7 +756,7 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>4.198</v>
+        <v>3.62</v>
       </c>
     </row>
     <row r="27">
@@ -765,7 +766,7 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.368</v>
+        <v>2.509</v>
       </c>
     </row>
     <row r="28">
@@ -775,7 +776,7 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>0.83</v>
+        <v>0.717</v>
       </c>
     </row>
     <row r="29">
@@ -785,7 +786,7 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>0.762</v>
+        <v>0.711</v>
       </c>
     </row>
     <row r="30">
@@ -795,7 +796,7 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>0.499</v>
+        <v>0.482</v>
       </c>
     </row>
     <row r="32">
@@ -805,7 +806,7 @@
         </is>
       </c>
       <c r="G32" t="n">
-        <v>83.248</v>
+        <v>85.601</v>
       </c>
     </row>
     <row r="33">
@@ -815,27 +816,27 @@
         </is>
       </c>
       <c r="G33" t="n">
-        <v>11.593</v>
+        <v>12.147</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Pinterest</t>
+          <t>Discord</t>
         </is>
       </c>
       <c r="G34" t="n">
-        <v>6.049</v>
+        <v>6</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Pinterest</t>
         </is>
       </c>
       <c r="G35" t="n">
-        <v>5.878</v>
+        <v>5.684</v>
       </c>
     </row>
     <row r="36">
@@ -845,7 +846,7 @@
         </is>
       </c>
       <c r="G36" t="n">
-        <v>1.952</v>
+        <v>2.149</v>
       </c>
     </row>
     <row r="38">
@@ -855,7 +856,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>0.123</v>
+        <v>0.142</v>
       </c>
     </row>
     <row r="39">
@@ -871,31 +872,31 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Panflix</t>
+          <t>UOL | Notícias em Tempo Real</t>
         </is>
       </c>
       <c r="H40" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>UOL | Notícias em Tempo Real</t>
+          <t>Folha de S.Paulo</t>
         </is>
       </c>
       <c r="H41" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.029</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Folha de S.Paulo</t>
+          <t>Brazilian Newspas</t>
         </is>
       </c>
       <c r="H42" t="n">
-        <v>0.019</v>
+        <v>0.025</v>
       </c>
     </row>
     <row r="44">
@@ -905,7 +906,7 @@
         </is>
       </c>
       <c r="I44" t="n">
-        <v>1.748</v>
+        <v>1.624</v>
       </c>
     </row>
     <row r="45">
@@ -915,7 +916,7 @@
         </is>
       </c>
       <c r="I45" t="n">
-        <v>0.826</v>
+        <v>0.771</v>
       </c>
     </row>
     <row r="46">
@@ -925,7 +926,7 @@
         </is>
       </c>
       <c r="I46" t="n">
-        <v>0.8070000000000001</v>
+        <v>0.737</v>
       </c>
     </row>
     <row r="47">
@@ -935,17 +936,17 @@
         </is>
       </c>
       <c r="I47" t="n">
-        <v>0.5580000000000001</v>
+        <v>0.405</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>ReadEra by READERA LLC</t>
+          <t>Bible</t>
         </is>
       </c>
       <c r="I48" t="n">
-        <v>0.375</v>
+        <v>0.34</v>
       </c>
     </row>
     <row r="50">
@@ -955,7 +956,7 @@
         </is>
       </c>
       <c r="J50" t="n">
-        <v>59.544</v>
+        <v>56.495</v>
       </c>
     </row>
     <row r="51">
@@ -965,7 +966,7 @@
         </is>
       </c>
       <c r="J51" t="n">
-        <v>26.815</v>
+        <v>26.608</v>
       </c>
     </row>
     <row r="52">
@@ -975,7 +976,7 @@
         </is>
       </c>
       <c r="J52" t="n">
-        <v>3.85</v>
+        <v>3.949</v>
       </c>
     </row>
     <row r="53">
@@ -985,7 +986,7 @@
         </is>
       </c>
       <c r="J53" t="n">
-        <v>2.577</v>
+        <v>2.839</v>
       </c>
     </row>
     <row r="54">
@@ -995,7 +996,7 @@
         </is>
       </c>
       <c r="J54" t="n">
-        <v>1.944</v>
+        <v>1.869</v>
       </c>
     </row>
     <row r="56">
@@ -1005,7 +1006,7 @@
         </is>
       </c>
       <c r="K56" t="n">
-        <v>9.939</v>
+        <v>10.135</v>
       </c>
     </row>
     <row r="57">
@@ -1015,7 +1016,7 @@
         </is>
       </c>
       <c r="K57" t="n">
-        <v>4.949</v>
+        <v>5.01</v>
       </c>
     </row>
     <row r="58">
@@ -1025,7 +1026,7 @@
         </is>
       </c>
       <c r="K58" t="n">
-        <v>0.997</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="59">
@@ -1035,17 +1036,17 @@
         </is>
       </c>
       <c r="K59" t="n">
-        <v>0.616</v>
+        <v>0.614</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Deezer</t>
+          <t>Music Player - MP3 Player, Audio Player</t>
         </is>
       </c>
       <c r="K60" t="n">
-        <v>0.24</v>
+        <v>0.247</v>
       </c>
     </row>
     <row r="62">
@@ -1055,7 +1056,7 @@
         </is>
       </c>
       <c r="L62" t="n">
-        <v>30.737</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="63">
@@ -1065,7 +1066,7 @@
         </is>
       </c>
       <c r="L63" t="n">
-        <v>6.081</v>
+        <v>6.98</v>
       </c>
     </row>
     <row r="64">
@@ -1075,7 +1076,7 @@
         </is>
       </c>
       <c r="L64" t="n">
-        <v>4.623</v>
+        <v>5.022</v>
       </c>
     </row>
     <row r="65">
@@ -1085,7 +1086,7 @@
         </is>
       </c>
       <c r="L65" t="n">
-        <v>3.285</v>
+        <v>3.81</v>
       </c>
     </row>
     <row r="66">
@@ -1095,7 +1096,7 @@
         </is>
       </c>
       <c r="L66" t="n">
-        <v>2.163</v>
+        <v>2.085</v>
       </c>
     </row>
     <row r="68">
@@ -1105,7 +1106,7 @@
         </is>
       </c>
       <c r="M68" t="n">
-        <v>15.561</v>
+        <v>13.872</v>
       </c>
     </row>
     <row r="69">
@@ -1115,7 +1116,7 @@
         </is>
       </c>
       <c r="M69" t="n">
-        <v>7.125</v>
+        <v>7.365</v>
       </c>
     </row>
     <row r="70">
@@ -1125,7 +1126,7 @@
         </is>
       </c>
       <c r="M70" t="n">
-        <v>3.644</v>
+        <v>3.045</v>
       </c>
     </row>
     <row r="71">
@@ -1135,7 +1136,7 @@
         </is>
       </c>
       <c r="M71" t="n">
-        <v>1.5</v>
+        <v>1.683</v>
       </c>
     </row>
     <row r="72">
@@ -1145,7 +1146,7 @@
         </is>
       </c>
       <c r="M72" t="n">
-        <v>1.072</v>
+        <v>1.048</v>
       </c>
     </row>
     <row r="74">
@@ -1155,7 +1156,7 @@
         </is>
       </c>
       <c r="N74" t="n">
-        <v>9.698</v>
+        <v>11.935</v>
       </c>
     </row>
     <row r="75">
@@ -1165,7 +1166,7 @@
         </is>
       </c>
       <c r="N75" t="n">
-        <v>4.952</v>
+        <v>5.592</v>
       </c>
     </row>
     <row r="76">
@@ -1175,7 +1176,7 @@
         </is>
       </c>
       <c r="N76" t="n">
-        <v>3.48</v>
+        <v>3.556</v>
       </c>
     </row>
     <row r="77">
@@ -1185,17 +1186,17 @@
         </is>
       </c>
       <c r="N77" t="n">
-        <v>3.053</v>
+        <v>3.152</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Uber Driver</t>
+          <t>Uber</t>
         </is>
       </c>
       <c r="N78" t="n">
-        <v>2.851</v>
+        <v>2.706</v>
       </c>
     </row>
     <row r="80">
@@ -1205,7 +1206,7 @@
         </is>
       </c>
       <c r="O80" t="n">
-        <v>14.344</v>
+        <v>13.947</v>
       </c>
     </row>
     <row r="81">
@@ -1215,7 +1216,7 @@
         </is>
       </c>
       <c r="O81" t="n">
-        <v>10.377</v>
+        <v>10.597</v>
       </c>
     </row>
     <row r="82">
@@ -1225,7 +1226,7 @@
         </is>
       </c>
       <c r="O82" t="n">
-        <v>5.595</v>
+        <v>5.877</v>
       </c>
     </row>
     <row r="83">
@@ -1235,7 +1236,7 @@
         </is>
       </c>
       <c r="O83" t="n">
-        <v>2.338</v>
+        <v>2.521</v>
       </c>
     </row>
     <row r="84">
@@ -1245,7 +1246,7 @@
         </is>
       </c>
       <c r="O84" t="n">
-        <v>1.761</v>
+        <v>2.042</v>
       </c>
     </row>
     <row r="86">
@@ -1255,40 +1256,90 @@
         </is>
       </c>
       <c r="B86" t="n">
-        <v>8.65</v>
+        <v>9.273</v>
       </c>
       <c r="E86" t="n">
-        <v>11.557</v>
+        <v>11.642</v>
       </c>
       <c r="F86" t="n">
-        <v>0.694</v>
+        <v>1.187</v>
       </c>
       <c r="G86" t="n">
-        <v>1.733</v>
+        <v>1.964</v>
       </c>
       <c r="H86" t="n">
-        <v>0.222</v>
+        <v>0.247</v>
       </c>
       <c r="I86" t="n">
-        <v>3.023</v>
+        <v>3.3</v>
       </c>
       <c r="J86" t="n">
-        <v>5.18</v>
+        <v>5.271</v>
       </c>
       <c r="K86" t="n">
-        <v>3.953</v>
+        <v>3.955</v>
       </c>
       <c r="L86" t="n">
-        <v>58.931</v>
+        <v>71.968</v>
       </c>
       <c r="M86" t="n">
-        <v>4.249</v>
+        <v>4.475</v>
       </c>
       <c r="N86" t="n">
-        <v>21.807</v>
+        <v>21.686</v>
       </c>
       <c r="O86" t="n">
-        <v>8.090999999999999</v>
+        <v>8.529999999999999</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>未分类 App</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>时长（十亿分钟）</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Google Play Store</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>4.267</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Mobitraxx PRO</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1.307</v>
       </c>
     </row>
   </sheetData>

</xml_diff>